<commit_message>
DATA. Entrenamiento parcial de modelos para USA y ENG con nueva preparacion de datos.
</commit_message>
<xml_diff>
--- a/data/argentina/p3_data_preparation/df_hiper_prep.xlsx
+++ b/data/argentina/p3_data_preparation/df_hiper_prep.xlsx
@@ -471,8 +471,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>30</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>[30, 180]</t>
+        </is>
       </c>
       <c r="B2" t="n">
         <v>3</v>
@@ -481,14 +483,14 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>

</xml_diff>